<commit_message>
updates changes to wadar
aanpassingen van de locatie tabel + andere kleine wadar aanpassingen
</commit_message>
<xml_diff>
--- a/mappings/locations-mapped.xlsx
+++ b/mappings/locations-mapped.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projecten\RWS\ISC-mapping-schelde\mappings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A254817B-1798-4398-88EA-A497787B55B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D15ACF8-2373-4B54-BC0B-E947A567A8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Identitication unique de la station</t>
   </si>
@@ -28,7 +28,7 @@
     <t>Localité</t>
   </si>
   <si>
-    <t>LOCOMS</t>
+    <t>locatie_code</t>
   </si>
   <si>
     <t>NL_HANSWGL</t>
@@ -37,9 +37,6 @@
     <t>Hansweert</t>
   </si>
   <si>
-    <t>Hansweert geul</t>
-  </si>
-  <si>
     <t>NL89_SASVGT</t>
   </si>
   <si>
@@ -58,31 +55,43 @@
     <t>Terneuzen</t>
   </si>
   <si>
-    <t>Terneuzen boei 20</t>
-  </si>
-  <si>
     <t>NL89_VLISSGBISSVH</t>
   </si>
   <si>
     <t>Vlissingen</t>
   </si>
   <si>
-    <t>Vlissingen boei SSVH</t>
-  </si>
-  <si>
     <t>NL95_WALCRN2</t>
   </si>
   <si>
     <t>Walcheren 2</t>
   </si>
   <si>
-    <t>Walcheren 2 km uit de kust</t>
-  </si>
-  <si>
     <t>NL89_WISSKKE</t>
   </si>
   <si>
     <t>Wissenkerke</t>
+  </si>
+  <si>
+    <t>hansweert.geul</t>
+  </si>
+  <si>
+    <t>sasvangent.grens</t>
+  </si>
+  <si>
+    <t>schaarvanoudendoel</t>
+  </si>
+  <si>
+    <t>terneuzen.boei20</t>
+  </si>
+  <si>
+    <t>vlissingen.boeissvh</t>
+  </si>
+  <si>
+    <t>walcheren.2kmuitdekust</t>
+  </si>
+  <si>
+    <t>wissenkerke</t>
   </si>
 </sst>
 </file>
@@ -446,14 +455,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.28515625" customWidth="1"/>
-    <col min="2" max="2" width="31.7109375" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -464,7 +472,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -472,73 +480,73 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B8" t="s">
         <v>16</v>
       </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>